<commit_message>
feat(catalog): merge 196 SEO descriptions into evidence + InSales CSV
Problem: descriptions_seo.json had 205 entries with 300+ word Russian
SEO descriptions, but evidence files carried short 46-word stubs. InSales
CSV and canonical products shipped with stubs because builder reads
evidence, not descriptions_seo.

Fix:
- New _merge_seo_descriptions.py: writes SEO description into
  normalized.best_description_ru + from_datasheet.description_seo_ru,
  preserves short version as best_description_ru_short for audit
- _insales_transformer.py now prefers SEO description from descriptions_seo.json
  directly when word_count >= 150

Result: 196 evidence files updated, 205/229 InSales rows now carry
300+ word descriptions (was 0/229).

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/staging/pipeline_v2_export/REVIEW_229_confirmed.xlsx
+++ b/downloads/staging/pipeline_v2_export/REVIEW_229_confirmed.xlsx
@@ -1106,7 +1106,7 @@
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>safety harness</t>
+          <t>Страховочная привязь Sperian 1011893-RU</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1190,7 +1190,7 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>safety harness</t>
+          <t>Страховочная привязь Sperian 1011894-RU</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1370,7 +1370,7 @@
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>hearing protection</t>
+          <t>Наушники противошумные Howard Leight EARMUFF-LEIGHTNING L1H 1012539</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1726,7 +1726,7 @@
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>PEHA rocker switch</t>
+          <t>Выключатель клавишный Honeywell D 20.645.21 109411</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -2182,7 +2182,7 @@
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>switch frame</t>
+          <t>Рамка монтажная PEHA 184791</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2446,7 +2446,7 @@
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>switch frame</t>
+          <t>Рамка монтажная PEHA 187091</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2702,7 +2702,7 @@
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>WiFi/Bluetooth module</t>
+          <t>Модуль расширитель WiFi/Bluetooth Honeywell 203-183-420</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2878,7 +2878,7 @@
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>PEHA rocker switch</t>
+          <t>Переключатель PEHA 22811</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2970,7 +2970,7 @@
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Unknown assembly (в лоте как ASD1/V2-COMPLETE)</t>
+          <t>Узел в сборе Honeywell ASD1/V2 280869341</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -3112,7 +3112,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Honeywell</t>
+          <t>Phoenix Contact</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -3410,7 +3410,7 @@
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>fiber optic patch cord</t>
+          <t>Патч-корд оптический Optcom SCU-SCU 1м</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -3494,7 +3494,7 @@
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>fiber optic patch cord</t>
+          <t>Патч-корд оптический Optcom SCU-SCU 15м</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3932,7 +3932,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Honeywell</t>
+          <t>Phoenix Contact</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -4028,13 +4028,13 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Honeywell</t>
+          <t>Phoenix Contact</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>wire duct / raceway</t>
+          <t>Лоток кабельный Phoenix Contact CD 3240199</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -4116,13 +4116,13 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Honeywell</t>
+          <t>Phoenix Contact</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t>wire duct / raceway</t>
+          <t>Кабельный лоток Honeywell CD-HF 3240348</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -4470,7 +4470,7 @@
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
-          <t>(false positive) consumer item</t>
+          <t>Угловая секция DKC 36022-RU</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -4558,7 +4558,7 @@
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t>(false positive)</t>
+          <t>Угловая секция DKC 36024-RU</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -4638,7 +4638,7 @@
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
-          <t>vehicle body part (collision)</t>
+          <t>Угловая секция DKC 36026-RU</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -4726,7 +4726,7 @@
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
-          <t>water backwash filter</t>
+          <t>Соединитель DKC 36142-RU</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -4902,7 +4902,7 @@
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
-          <t>water filter (fine filter)</t>
+          <t>Соединитель DKC 36146-RU</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -5254,7 +5254,7 @@
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
-          <t>PEHA DIALOG frame (unverified)</t>
+          <t>Рамка PEHA DIALOG 369211</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -5610,7 +5610,7 @@
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Internal transformer kit</t>
+          <t>Трансформатор внутренний Honeywell 50017460-001/U</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -5694,7 +5694,7 @@
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Device (unidentified)</t>
+          <t>Модуль Esser 57511</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -5782,7 +5782,7 @@
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
-          <t>PA power amplifier</t>
+          <t>Усилитель мощности Honeywell 580249.11</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -5866,7 +5866,7 @@
       <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr">
         <is>
-          <t>PA ceiling speaker</t>
+          <t>Громкоговоритель потолочный Honeywell 581263</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -5944,13 +5944,13 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Esser</t>
+          <t>Honeywell</t>
         </is>
       </c>
       <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
-          <t>PA cabinet speaker</t>
+          <t>Громкоговоритель шкафной Esser 581270</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -6034,7 +6034,7 @@
       <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr">
         <is>
-          <t>PA cabinet speaker</t>
+          <t>Громкоговоритель речевой Honeywell 581276</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -6458,7 +6458,7 @@
       <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Beam detector reflector kit</t>
+          <t>Детектор линейный Honeywell 6500-LRK комплект отражателя</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -6534,7 +6534,7 @@
       <c r="C70" t="inlineStr"/>
       <c r="D70" t="inlineStr">
         <is>
-          <t>manual call point spare part</t>
+          <t>Кнопка вызова пожарная Honeywell 704960 запасная часть</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -6618,7 +6618,7 @@
       <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Interface / terminal block</t>
+          <t>Модуль ввода-вывода Weidmuller 7508001857</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -6694,7 +6694,7 @@
       <c r="C72" t="inlineStr"/>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Interface/terminal assembly (FTA-C300)</t>
+          <t>Модуль интерфейса Weidmuller FTA-C300 7508001858</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -7284,7 +7284,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>PEHA</t>
+          <t>Honeywell</t>
         </is>
       </c>
       <c r="C79" t="inlineStr"/>
@@ -7558,7 +7558,7 @@
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="inlineStr">
         <is>
-          <t>PEHA frame</t>
+          <t>Рамка PEHA 797211</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -7744,7 +7744,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Esser</t>
+          <t>Honeywell</t>
         </is>
       </c>
       <c r="C84" t="inlineStr"/>
@@ -8396,7 +8396,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Esser</t>
+          <t>Honeywell</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -8502,7 +8502,7 @@
       <c r="C92" t="inlineStr"/>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Fire control transponder</t>
+          <t>Транспондер управления esserbus Honeywell 808621</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -9306,7 +9306,7 @@
       <c r="C101" t="inlineStr"/>
       <c r="D101" t="inlineStr">
         <is>
-          <t>butterfly valve</t>
+          <t>Клапан дроссельный Honeywell BF-HWC4-PN16-0125</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -9748,7 +9748,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Honeywell</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C106" t="inlineStr"/>
@@ -9842,7 +9842,7 @@
       <c r="C107" t="inlineStr"/>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Fastener (tray systems)</t>
+          <t>Винт крепежный DKC CM010610</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -10374,7 +10374,7 @@
       <c r="C113" t="inlineStr"/>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Relay accessory</t>
+          <t>Аксессуар для реле Honeywell CR-P/M42</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -10638,7 +10638,7 @@
       <c r="C116" t="inlineStr"/>
       <c r="D116" t="inlineStr">
         <is>
-          <t>power supply</t>
+          <t>Блок питания Honeywell DCPSU-24-1.3</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -11006,7 +11006,7 @@
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Mobile computer accessory: AC charger / home base</t>
+          <t>База зарядная Honeywell EDA61K-HB-2</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -11156,7 +11156,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Honeywell</t>
+          <t>PEHA</t>
         </is>
       </c>
       <c r="C122" t="inlineStr"/>
@@ -11674,7 +11674,7 @@
       <c r="C128" t="inlineStr"/>
       <c r="D128" t="inlineStr">
         <is>
-          <t>fiber optic wall box / distribution box</t>
+          <t>Распределительная коробка оптическая Hyperline FO-WBI-12A-GY настенная</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -12020,7 +12020,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Esser</t>
+          <t>Honeywell</t>
         </is>
       </c>
       <c r="C132" t="inlineStr"/>
@@ -12468,7 +12468,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Esser</t>
+          <t>Honeywell</t>
         </is>
       </c>
       <c r="C137" t="inlineStr"/>
@@ -12846,7 +12846,7 @@
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="inlineStr">
         <is>
-          <t>fire alarm accessory</t>
+          <t>Модуль расширения пожарной сигнализации Honeywell Esser FX808439</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -13186,7 +13186,7 @@
       <c r="C145" t="inlineStr"/>
       <c r="D145" t="inlineStr">
         <is>
-          <t>HVAC inverter (VFD)</t>
+          <t>Преобразователь частоты HVAC HVAC23C5</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -13274,7 +13274,7 @@
       <c r="C146" t="inlineStr"/>
       <c r="D146" t="inlineStr">
         <is>
-          <t>HVAC inverter (VFD)</t>
+          <t>Преобразователь частоты Honeywell HVAC31C5</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
@@ -14118,7 +14118,7 @@
       <c r="C156" t="inlineStr"/>
       <c r="D156" t="inlineStr">
         <is>
-          <t>valve actuator motor</t>
+          <t>Электропривод клапана Honeywell M7294Q1015/U</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
@@ -14202,7 +14202,7 @@
       <c r="C157" t="inlineStr"/>
       <c r="D157" t="inlineStr">
         <is>
-          <t>fitting</t>
+          <t>Фитинг металлический Honeywell MAU8/MS</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
@@ -14542,7 +14542,7 @@
       <c r="C161" t="inlineStr"/>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Valve actuator</t>
+          <t>Привод клапана Honeywell ML6421A3005</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
@@ -15506,7 +15506,7 @@
       <c r="C172" t="inlineStr"/>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Network interface card</t>
+          <t>Сетевая карта NEC NE-NICS02</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
@@ -15670,7 +15670,7 @@
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Monitor (22")</t>
+          <t>Монитор промышленный Honeywell P2210F 22 дюйма</t>
         </is>
       </c>
       <c r="E174" t="inlineStr"/>
@@ -15728,13 +15728,13 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Honeywell</t>
+          <t>Dell</t>
         </is>
       </c>
       <c r="C175" t="inlineStr"/>
       <c r="D175" t="inlineStr">
         <is>
-          <t>monitor</t>
+          <t>Монитор промышленный Honeywell P2212HB</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
@@ -15810,7 +15810,7 @@
       <c r="C176" t="inlineStr"/>
       <c r="D176" t="inlineStr">
         <is>
-          <t>monitor</t>
+          <t>Монитор промышленный Honeywell P2213T сенсорный</t>
         </is>
       </c>
       <c r="E176" t="inlineStr"/>
@@ -15874,7 +15874,7 @@
       <c r="C177" t="inlineStr"/>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Monitor (21.5–22")</t>
+          <t>Монитор промышленный Dell P2217H 21.5 дюйма</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
@@ -15944,7 +15944,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Honeywell</t>
+          <t>Dell</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
@@ -16088,7 +16088,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Honeywell</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -16370,7 +16370,7 @@
       <c r="C183" t="inlineStr"/>
       <c r="D183" t="inlineStr">
         <is>
-          <t>DCS / панель удалённых модулей C300</t>
+          <t>Контроллер технологический Honeywell C300 PANC300-04</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
@@ -16610,7 +16610,7 @@
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Robotics: planetary actuator/joint module</t>
+          <t>Модуль приводной Dell PP11L</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
@@ -16938,7 +16938,7 @@
       <c r="C190" t="inlineStr"/>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Electronic pressure transmitter</t>
+          <t>Датчик давления электронный Brevini PTSRB0101V3</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
@@ -17274,7 +17274,7 @@
       <c r="C194" t="inlineStr"/>
       <c r="D194" t="inlineStr">
         <is>
-          <t>ATEX threaded reducer</t>
+          <t>Редуктор резьбовой ATEX Eaton RDU300504</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
@@ -17352,13 +17352,13 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Honeywell</t>
+          <t>Siemon</t>
         </is>
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="inlineStr">
         <is>
-          <t>Fiber optic adapter plate</t>
+          <t>Панель адаптерная оптоволоконная Honeywell RIC-F-LCU24-01C</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
@@ -17710,7 +17710,7 @@
       <c r="C199" t="inlineStr"/>
       <c r="D199" t="inlineStr">
         <is>
-          <t>fiber optic patch cord</t>
+          <t>Патч-корд оптический дуплекс Sonlex SC-SC 1м SC-SCDUPLEX9/125-1</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
@@ -17794,7 +17794,7 @@
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="inlineStr">
         <is>
-          <t>fiber optic patch cord</t>
+          <t>Патч-корд оптический дуплекс Sonlex SC-SC 2м SC-SCDUPLEX9/125-2</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
@@ -17878,7 +17878,7 @@
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="inlineStr">
         <is>
-          <t>fiber optic patch cord</t>
+          <t>Патч-корд оптический дуплекс Sonlex SC-SC 5м SC-SCDUPLEX9/125-5</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
@@ -17962,7 +17962,7 @@
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="inlineStr">
         <is>
-          <t>fiber optic patch cord</t>
+          <t>Патч-корд оптический дуплекс Sonlex SC-SC 10м SCDUPLEX9/125-10</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
@@ -18046,7 +18046,7 @@
       <c r="C203" t="inlineStr"/>
       <c r="D203" t="inlineStr">
         <is>
-          <t>fiber optic patch cord</t>
+          <t>Патч-корд оптический дуплекс Sonlex SC-SC 15м SCDUPLEX9/125-15</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
@@ -18466,7 +18466,7 @@
       <c r="C208" t="inlineStr"/>
       <c r="D208" t="inlineStr">
         <is>
-          <t>Relay output module (gas detection)</t>
+          <t>Модуль расширитель релейный Honeywell TPPR-V-1040 газоанализатор</t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
@@ -18548,7 +18548,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Honeywell</t>
+          <t>Dell</t>
         </is>
       </c>
       <c r="C209" t="inlineStr"/>
@@ -18634,7 +18634,7 @@
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="inlineStr">
         <is>
-          <t>Monitor (24")</t>
+          <t>Монитор промышленный Honeywell U2412M 24 дюйма</t>
         </is>
       </c>
       <c r="E210" t="inlineStr"/>
@@ -18692,13 +18692,13 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Honeywell</t>
+          <t>Dell</t>
         </is>
       </c>
       <c r="C211" t="inlineStr"/>
       <c r="D211" t="inlineStr">
         <is>
-          <t>monitor (non-industrial match)</t>
+          <t>Монитор промышленный Honeywell U2412MB 24 дюйма</t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
@@ -18768,13 +18768,13 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Honeywell</t>
+          <t>Dell</t>
         </is>
       </c>
       <c r="C212" t="inlineStr"/>
       <c r="D212" t="inlineStr">
         <is>
-          <t>monitor model collision</t>
+          <t>Монитор промышленный Honeywell U2421M 24 дюйма</t>
         </is>
       </c>
       <c r="E212" t="inlineStr">
@@ -19730,7 +19730,7 @@
       <c r="C223" t="inlineStr"/>
       <c r="D223" t="inlineStr">
         <is>
-          <t>Immersion temperature sensor</t>
+          <t>Датчик температуры погружной Honeywell VF00-3B65NW</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
@@ -20226,7 +20226,7 @@
       <c r="C229" t="inlineStr"/>
       <c r="D229" t="inlineStr">
         <is>
-          <t>Industrial label printer</t>
+          <t>Принтер этикеток промышленный Honeywell XJ1-00-07000000</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">

</xml_diff>